<commit_message>
Excel: add verified findings from Bertolini 2009, API 581 Add.1 Part 1 s8 and ASME PCC-3-2022; correct Bertolini description
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014T3x3vbmLmpBHxXp5vGwhE
</commit_message>
<xml_diff>
--- a/Barrancabermeja_RBI/DSS_RBI_Barrancabermeja_UNA_HOJA.xlsx
+++ b/Barrancabermeja_RBI/DSS_RBI_Barrancabermeja_UNA_HOJA.xlsx
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1444" uniqueCount="894">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1452" uniqueCount="902">
   <si>
     <t xml:space="preserve">DSS RBI – Beneficios económicos por reducción de riesgo · Barrancabermeja (UNA HOJA)</t>
   </si>
@@ -2440,6 +2440,24 @@
     <t xml:space="preserve">19 · AUDITORÍA, INVENTARIO, BIBLIOGRAFÍA, NORMAS, RESPUESTAS Y PENDIENTES</t>
   </si>
   <si>
+    <t xml:space="preserve">19.0 Verificado con los adjuntos (Bertolini 2009; API 581 Adenda 1 abr-2019 Parte 1 §8; ASME PCC-3-2022)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API 581 Parte 1 §8, ejemplo 8.4.2: Cf = 25 %·100.000·4/100 + 25.000 + 25.000 + 0 = 150.000 $ (Eq. 1.65) ✓; Pf,max = 75.000/150.000 = 0,5 (Eq. 1.68) ✓; ejemplo de inspección: tasa = (0,12−0,104)/11,75 = 0,001362 in/a (1.71) y PBL_adj = 0,5·0,12/0,001362 = 44,1 años (1.72) ✓ recalculados. No reproduje los 7,1 y 17,1 años (la aplicación de la incertidumbre AU 50 %/30 % no queda clara en el texto).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API 581 Parte 1 §8.6.4: una inspección no reduce el riesgo por sí misma; reduce la incertidumbre y conoce la condición real (curva Weibull se desplaza). §8.7.2: decisión inspeccionar/reemplazar comparando costo de la acción con el riesgo incremental por diferir (Eqs. 1.78–1.80). El texto dice "En la Ecuación (1.80), t1…" (debe ser 1.78) y la nomenclatura da EIR en $/año aunque la ecuación da $ por intervalo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API 581 Parte 1 §8.1.4/8.3.3: los módulos usan una biblioteca de confiabilidad (Weibayes). Es la ruta API para haces; la coraza (Oropallo) usa gff·Df·FMS. Un intercambiador de tubo y coraza requiere ambos módulos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASME PCC-3-2022: es una guía de planificación; define cualitativo/semicuantitativo/cuantitativo como continuo (Fig. 3.3.1-1), 6 niveles de probabilidad (§7.3) y de pérdida económica (Tabla 8.3.7-1), matriz de ejemplo (Fig. 9.5.1-1) y gráfico NPVS (§9.5.3). No contiene ecuaciones de POF ni de VAN.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bertolini 2009 (leído): J-factor = (riesgo original − nuevo)/costo, sin descuento y con riesgo en puntaje de matriz; ver 19.3.</t>
+  </si>
+  <si>
     <t xml:space="preserve">19.1 Auditoría del paper (inconsistencias)</t>
   </si>
   <si>
@@ -2596,7 +2614,7 @@
     <t xml:space="preserve">19.3 Bibliografía: 3 referencias más relevantes (+ suplentes)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Bertolini, Bevilacqua, Ciarapica, Giacchetta (2009) 'Development of risk-based inspection and maintenance procedures for an oil refinery'. J. Loss Prev. Process Ind. 22(2), 244–253. — https://doi.org/10.1016/j.jlp.2009.01.003 — Es el referente más cercano a Barrancabermeja: RBI aplicado a una refinería con análisis económico de procedimientos. Oropallo lo cita (p.4, p.5) para reducción de recursos de inspección, ampliación de intervalos y menos paros. Aporta: estructura refinería → equipos → plan → beneficio.</t>
+    <t xml:space="preserve">1. Bertolini, Bevilacqua, Ciarapica, Giacchetta (2009) 'Development of risk-based inspection and maintenance procedures for an oil refinery'. J. Loss Prev. Process Ind. 22(2), 244–253. — https://doi.org/10.1016/j.jlp.2009.01.003 — LEÍDO. Procedimiento RBI&amp;M de 6 módulos (panel Delphi de 15 expertos, refinería de Ancona, 3,9 Mt/año): matriz 5×5 (probabilidad A–E × severidad 1–5 con 4 impactos: seguridad, ambiente, reputación y económico &lt;10 k€ … &gt;10 M€), riesgo = probabilidad × exposición × consecuencia, y J-factor = (riesgo original − riesgo nuevo)/costo. Resultados (Tabla 5): horas −20 %/−14 %, costos −18 %/−9 %; partidas en parada −23 % (2004) y −9,5 % (2005). NO usa API 581 ni VAN y su 'riesgo' es un puntaje de matriz, no dólares. Aporta: matriz multi-impacto, J-factor como antecedente del SIR y evidencia de ahorros en refinería. Corrige mi descripción previa ('análisis económico'), que era excesiva.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Khan &amp; Haddara (2004) 'Risk-Based Maintenance (RBM): a new approach for process plant inspection and maintenance'. Process Saf. Prog. 23(4), 252–265. — https://doi.org/10.1002/prs.10010 — Base conceptual de riesgo = PoF×CoF como costo esperado y de la optimización del intervalo de inspección (mínimo de costo de inspección + riesgo). Sostiene el núcleo ΔEMV y la decisión de 'cuándo inspeccionar'.</t>
@@ -2611,7 +2629,7 @@
     <t xml:space="preserve">Alt.. Rodríguez-Prieto, Camacho, Callejas, Sebastián (2020) 'Fitness for service and reliability of materials… petrochemical industry'. IEEE Access 8, 92275–92286. — https://doi.org/10.1109/ACCESS.2020.2994619 — Suplente: vínculo FFS–confiabilidad en petroquímica (útil para V-220).</t>
   </si>
   <si>
-    <t xml:space="preserve">Los DOI/enlaces se tomaron de la bibliografía del PDF de Oropallo (verificado). Las referencias NO se abrieron en esta sesión (sin acceso a editoriales): su aporte se describe por el contexto en que las cita Oropallo y por conocimiento general del agente → PENDIENTE de lectura.</t>
+    <t xml:space="preserve">Los DOI se tomaron de la bibliografía del PDF de Oropallo (verificado). Bertolini et al. (2009) fue leído completo; Khan &amp; Haddara (2004) y Straub &amp; Faber (2005) NO se han leído: su aporte se describe por el contexto en que los cita Oropallo → PENDIENTE de lectura.</t>
   </si>
   <si>
     <t xml:space="preserve">19.4 Verificación de normas (ubicación exacta: verificada vs probable)</t>
@@ -2644,7 +2662,13 @@
     <t xml:space="preserve">Adenda(s) 2018–2020 sobre CA · API RP 581 · Fuentes públicas indican: Adenda 2 (emitida 1-oct-2020 según la tienda) modifica Partes incl. CA; resumen público: se elimina el límite de 10.000 ft² en COF Nivel 1 y 2. Existe además un documento fechado abril 2019. NO se pudo abrir el texto · Estado: PENDIENTE · Acción: Leer el texto de las adendas; no afirmar cuál adenda contiene cada cambio</t>
   </si>
   <si>
-    <t xml:space="preserve">Claves de un programa RBI; 'shall' vs 'should'; continuum · API RP 580 · Conocimiento técnico: elementos clave (sistema de gestión, método documentado de PoF, método de CoF, método de gestión del riesgo); continuo cualitativo→cuantitativo; 'shall'=requisito mínimo, 'should'=recomendación · Estado: Conocimiento: PENDIENTE de validación · Acción: Verificar Secciones 1 y 7 / prefacio de API 580 (ed. aplicable)</t>
+    <t xml:space="preserve">Continuum de enfoques; shall/should/may · ASME PCC-3-2022 (leído) · API 580 (no disponible) · PCC-3 Foreword: 'shall' = requisito, 'should' = recomendación, 'may' = permiso. PCC-3 §3.3 y Fig. 3.3.1-1 'Continuum of RBI Approaches' (cualitativo – semicuantitativo – cuantitativo); §3.3.4: los enfoques son complementarios, no competidores · Estado: PCC-3: VERIFICADO · API 580: PENDIENTE de validación · Acción: Verificar la convención y las claves de un programa en API 580 (ed. aplicable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCC-3 §7–10 (POF, COF, riesgo, gestión con inspección) · ASME PCC-3-2022 (leído) · §7 Determining POF (categorías de 3 y 6 niveles, §7.3); §8 Determining COF (§8.3.6–8.3.7: costo de oportunidad = valor diario de la unidad × días de paro; Tabla 8.3.7-1 de 6 niveles de pérdida económica); §9 (Fig. 9.5.1-1 matriz de ejemplo; §9.5.3 gráfico de ahorro de valor presente neto vs tiempo de inspección); §10.1 la inspección no detiene el daño: reduce incertidumbre. PCC-3 NO trae la ecuación POF=gff·Df·FMS · Estado: VERIFICADO · Acción: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">API 581 Adenda 1 (abril 2019) Parte 1 §8 Haces de intercambiadores · API RP 581 3.ª ed. 2016 + Adenda 1 (leído, pp. 1-86 a 1-102) · POF del haz por Weibull (Eq. 1.54–1.61, 1.74–1.77); Cf=Cost_prod+Cost_env+Cost_bundle+Cost_maint (1.62); Cost_prod=Unit·D_sd·Rate_red/100 (1.63); Riesgo=Pf·Cf (1.66); Pf,max=Risk_tgt/Cf (1.67); riesgo incremental esperado por diferir EIR=Cf·(1−[1−Pf(t2)]/[1−Pf(t1)]) (1.78); inspeccionar si (Cost_insp+Cost_maint)(1+ROR)&lt;EIR (1.79); reemplazar (1.80); frecuencia óptima de reemplazo minimizando costo total (1.81–1.89). Matriz de riesgo: Parte 1 Figs. 4.2 y 4.3 y Tabla 8.7 (por referencia cruzada) · Estado: VERIFICADO (módulo de haces; la POF de la coraza con Df NO está en este extracto) · Acción: Las Eqs. 1.78–1.80 son la base API de 'ahorro por diferimiento'</t>
   </si>
   <si>
     <t xml:space="preserve">FFS Niveles 1–3 · API 579-1/ASME FFS-1 · Nivel 3 = análisis detallado (FEA elasto-plástico); Partes 4 (GML), 5 (LTA), 6 (picaduras) … · Estado: Conocimiento: PENDIENTE de validación · Acción: Verificar partes y criterios (RSF, MAWP reducida)</t>
@@ -3418,7 +3442,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AR686"/>
+  <dimension ref="A1:AR695"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -24664,7 +24688,7 @@
       <c r="O571" s="42"/>
       <c r="P571" s="42"/>
     </row>
-    <row r="572" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="572" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A572" s="5" t="s">
         <v>784</v>
       </c>
@@ -24684,7 +24708,7 @@
       <c r="O572" s="5"/>
       <c r="P572" s="5"/>
     </row>
-    <row r="573" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="573" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A573" s="5" t="s">
         <v>785</v>
       </c>
@@ -24704,7 +24728,7 @@
       <c r="O573" s="5"/>
       <c r="P573" s="5"/>
     </row>
-    <row r="574" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="574" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A574" s="5" t="s">
         <v>786</v>
       </c>
@@ -24764,49 +24788,29 @@
       <c r="O576" s="5"/>
       <c r="P576" s="5"/>
     </row>
-    <row r="577" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A577" s="5" t="s">
+    <row r="578" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A578" s="42" t="s">
         <v>789</v>
       </c>
-      <c r="B577" s="5"/>
-      <c r="C577" s="5"/>
-      <c r="D577" s="5"/>
-      <c r="E577" s="5"/>
-      <c r="F577" s="5"/>
-      <c r="G577" s="5"/>
-      <c r="H577" s="5"/>
-      <c r="I577" s="5"/>
-      <c r="J577" s="5"/>
-      <c r="K577" s="5"/>
-      <c r="L577" s="5"/>
-      <c r="M577" s="5"/>
-      <c r="N577" s="5"/>
-      <c r="O577" s="5"/>
-      <c r="P577" s="5"/>
-    </row>
-    <row r="578" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A578" s="5" t="s">
-        <v>790</v>
-      </c>
-      <c r="B578" s="5"/>
-      <c r="C578" s="5"/>
-      <c r="D578" s="5"/>
-      <c r="E578" s="5"/>
-      <c r="F578" s="5"/>
-      <c r="G578" s="5"/>
-      <c r="H578" s="5"/>
-      <c r="I578" s="5"/>
-      <c r="J578" s="5"/>
-      <c r="K578" s="5"/>
-      <c r="L578" s="5"/>
-      <c r="M578" s="5"/>
-      <c r="N578" s="5"/>
-      <c r="O578" s="5"/>
-      <c r="P578" s="5"/>
+      <c r="B578" s="42"/>
+      <c r="C578" s="42"/>
+      <c r="D578" s="42"/>
+      <c r="E578" s="42"/>
+      <c r="F578" s="42"/>
+      <c r="G578" s="42"/>
+      <c r="H578" s="42"/>
+      <c r="I578" s="42"/>
+      <c r="J578" s="42"/>
+      <c r="K578" s="42"/>
+      <c r="L578" s="42"/>
+      <c r="M578" s="42"/>
+      <c r="N578" s="42"/>
+      <c r="O578" s="42"/>
+      <c r="P578" s="42"/>
     </row>
     <row r="579" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A579" s="5" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B579" s="5"/>
       <c r="C579" s="5"/>
@@ -24826,7 +24830,7 @@
     </row>
     <row r="580" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A580" s="5" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B580" s="5"/>
       <c r="C580" s="5"/>
@@ -24846,7 +24850,7 @@
     </row>
     <row r="581" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A581" s="5" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B581" s="5"/>
       <c r="C581" s="5"/>
@@ -24864,9 +24868,9 @@
       <c r="O581" s="5"/>
       <c r="P581" s="5"/>
     </row>
-    <row r="582" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="582" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A582" s="5" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B582" s="5"/>
       <c r="C582" s="5"/>
@@ -24886,7 +24890,7 @@
     </row>
     <row r="583" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A583" s="5" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B583" s="5"/>
       <c r="C583" s="5"/>
@@ -24904,9 +24908,9 @@
       <c r="O583" s="5"/>
       <c r="P583" s="5"/>
     </row>
-    <row r="584" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="584" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A584" s="5" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="B584" s="5"/>
       <c r="C584" s="5"/>
@@ -24926,7 +24930,7 @@
     </row>
     <row r="585" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A585" s="5" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="B585" s="5"/>
       <c r="C585" s="5"/>
@@ -24946,7 +24950,7 @@
     </row>
     <row r="586" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A586" s="5" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B586" s="5"/>
       <c r="C586" s="5"/>
@@ -24964,9 +24968,9 @@
       <c r="O586" s="5"/>
       <c r="P586" s="5"/>
     </row>
-    <row r="587" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="587" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A587" s="5" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B587" s="5"/>
       <c r="C587" s="5"/>
@@ -24986,7 +24990,7 @@
     </row>
     <row r="588" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A588" s="5" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="B588" s="5"/>
       <c r="C588" s="5"/>
@@ -25004,25 +25008,45 @@
       <c r="O588" s="5"/>
       <c r="P588" s="5"/>
     </row>
+    <row r="589" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A589" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="B589" s="5"/>
+      <c r="C589" s="5"/>
+      <c r="D589" s="5"/>
+      <c r="E589" s="5"/>
+      <c r="F589" s="5"/>
+      <c r="G589" s="5"/>
+      <c r="H589" s="5"/>
+      <c r="I589" s="5"/>
+      <c r="J589" s="5"/>
+      <c r="K589" s="5"/>
+      <c r="L589" s="5"/>
+      <c r="M589" s="5"/>
+      <c r="N589" s="5"/>
+      <c r="O589" s="5"/>
+      <c r="P589" s="5"/>
+    </row>
     <row r="590" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A590" s="42" t="s">
+      <c r="A590" s="5" t="s">
         <v>801</v>
       </c>
-      <c r="B590" s="42"/>
-      <c r="C590" s="42"/>
-      <c r="D590" s="42"/>
-      <c r="E590" s="42"/>
-      <c r="F590" s="42"/>
-      <c r="G590" s="42"/>
-      <c r="H590" s="42"/>
-      <c r="I590" s="42"/>
-      <c r="J590" s="42"/>
-      <c r="K590" s="42"/>
-      <c r="L590" s="42"/>
-      <c r="M590" s="42"/>
-      <c r="N590" s="42"/>
-      <c r="O590" s="42"/>
-      <c r="P590" s="42"/>
+      <c r="B590" s="5"/>
+      <c r="C590" s="5"/>
+      <c r="D590" s="5"/>
+      <c r="E590" s="5"/>
+      <c r="F590" s="5"/>
+      <c r="G590" s="5"/>
+      <c r="H590" s="5"/>
+      <c r="I590" s="5"/>
+      <c r="J590" s="5"/>
+      <c r="K590" s="5"/>
+      <c r="L590" s="5"/>
+      <c r="M590" s="5"/>
+      <c r="N590" s="5"/>
+      <c r="O590" s="5"/>
+      <c r="P590" s="5"/>
     </row>
     <row r="591" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A591" s="5" t="s">
@@ -25084,7 +25108,7 @@
       <c r="O593" s="5"/>
       <c r="P593" s="5"/>
     </row>
-    <row r="594" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="594" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A594" s="5" t="s">
         <v>805</v>
       </c>
@@ -25124,49 +25148,29 @@
       <c r="O595" s="5"/>
       <c r="P595" s="5"/>
     </row>
-    <row r="596" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A596" s="5" t="s">
+    <row r="597" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A597" s="42" t="s">
         <v>807</v>
       </c>
-      <c r="B596" s="5"/>
-      <c r="C596" s="5"/>
-      <c r="D596" s="5"/>
-      <c r="E596" s="5"/>
-      <c r="F596" s="5"/>
-      <c r="G596" s="5"/>
-      <c r="H596" s="5"/>
-      <c r="I596" s="5"/>
-      <c r="J596" s="5"/>
-      <c r="K596" s="5"/>
-      <c r="L596" s="5"/>
-      <c r="M596" s="5"/>
-      <c r="N596" s="5"/>
-      <c r="O596" s="5"/>
-      <c r="P596" s="5"/>
-    </row>
-    <row r="597" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A597" s="5" t="s">
-        <v>808</v>
-      </c>
-      <c r="B597" s="5"/>
-      <c r="C597" s="5"/>
-      <c r="D597" s="5"/>
-      <c r="E597" s="5"/>
-      <c r="F597" s="5"/>
-      <c r="G597" s="5"/>
-      <c r="H597" s="5"/>
-      <c r="I597" s="5"/>
-      <c r="J597" s="5"/>
-      <c r="K597" s="5"/>
-      <c r="L597" s="5"/>
-      <c r="M597" s="5"/>
-      <c r="N597" s="5"/>
-      <c r="O597" s="5"/>
-      <c r="P597" s="5"/>
+      <c r="B597" s="42"/>
+      <c r="C597" s="42"/>
+      <c r="D597" s="42"/>
+      <c r="E597" s="42"/>
+      <c r="F597" s="42"/>
+      <c r="G597" s="42"/>
+      <c r="H597" s="42"/>
+      <c r="I597" s="42"/>
+      <c r="J597" s="42"/>
+      <c r="K597" s="42"/>
+      <c r="L597" s="42"/>
+      <c r="M597" s="42"/>
+      <c r="N597" s="42"/>
+      <c r="O597" s="42"/>
+      <c r="P597" s="42"/>
     </row>
     <row r="598" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A598" s="5" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B598" s="5"/>
       <c r="C598" s="5"/>
@@ -25186,7 +25190,7 @@
     </row>
     <row r="599" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A599" s="5" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B599" s="5"/>
       <c r="C599" s="5"/>
@@ -25206,7 +25210,7 @@
     </row>
     <row r="600" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A600" s="5" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B600" s="5"/>
       <c r="C600" s="5"/>
@@ -25226,7 +25230,7 @@
     </row>
     <row r="601" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A601" s="5" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B601" s="5"/>
       <c r="C601" s="5"/>
@@ -25246,7 +25250,7 @@
     </row>
     <row r="602" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A602" s="5" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B602" s="5"/>
       <c r="C602" s="5"/>
@@ -25266,7 +25270,7 @@
     </row>
     <row r="603" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A603" s="5" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B603" s="5"/>
       <c r="C603" s="5"/>
@@ -25286,7 +25290,7 @@
     </row>
     <row r="604" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A604" s="5" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B604" s="5"/>
       <c r="C604" s="5"/>
@@ -25306,7 +25310,7 @@
     </row>
     <row r="605" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A605" s="5" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="B605" s="5"/>
       <c r="C605" s="5"/>
@@ -25326,7 +25330,7 @@
     </row>
     <row r="606" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A606" s="5" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B606" s="5"/>
       <c r="C606" s="5"/>
@@ -25346,7 +25350,7 @@
     </row>
     <row r="607" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A607" s="5" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="B607" s="5"/>
       <c r="C607" s="5"/>
@@ -25366,7 +25370,7 @@
     </row>
     <row r="608" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A608" s="5" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B608" s="5"/>
       <c r="C608" s="5"/>
@@ -25386,7 +25390,7 @@
     </row>
     <row r="609" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A609" s="5" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B609" s="5"/>
       <c r="C609" s="5"/>
@@ -25406,7 +25410,7 @@
     </row>
     <row r="610" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A610" s="5" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B610" s="5"/>
       <c r="C610" s="5"/>
@@ -25426,7 +25430,7 @@
     </row>
     <row r="611" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A611" s="5" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B611" s="5"/>
       <c r="C611" s="5"/>
@@ -25446,7 +25450,7 @@
     </row>
     <row r="612" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A612" s="5" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="B612" s="5"/>
       <c r="C612" s="5"/>
@@ -25466,7 +25470,7 @@
     </row>
     <row r="613" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A613" s="5" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B613" s="5"/>
       <c r="C613" s="5"/>
@@ -25486,7 +25490,7 @@
     </row>
     <row r="614" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A614" s="5" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B614" s="5"/>
       <c r="C614" s="5"/>
@@ -25506,7 +25510,7 @@
     </row>
     <row r="615" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A615" s="5" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="B615" s="5"/>
       <c r="C615" s="5"/>
@@ -25524,9 +25528,9 @@
       <c r="O615" s="5"/>
       <c r="P615" s="5"/>
     </row>
-    <row r="616" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="616" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A616" s="5" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="B616" s="5"/>
       <c r="C616" s="5"/>
@@ -25546,7 +25550,7 @@
     </row>
     <row r="617" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A617" s="5" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="B617" s="5"/>
       <c r="C617" s="5"/>
@@ -25566,7 +25570,7 @@
     </row>
     <row r="618" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A618" s="5" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="B618" s="5"/>
       <c r="C618" s="5"/>
@@ -25586,7 +25590,7 @@
     </row>
     <row r="619" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A619" s="5" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="B619" s="5"/>
       <c r="C619" s="5"/>
@@ -25606,7 +25610,7 @@
     </row>
     <row r="620" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A620" s="5" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="B620" s="5"/>
       <c r="C620" s="5"/>
@@ -25624,9 +25628,9 @@
       <c r="O620" s="5"/>
       <c r="P620" s="5"/>
     </row>
-    <row r="621" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="621" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A621" s="5" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="B621" s="5"/>
       <c r="C621" s="5"/>
@@ -25644,9 +25648,9 @@
       <c r="O621" s="5"/>
       <c r="P621" s="5"/>
     </row>
-    <row r="622" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="622" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A622" s="5" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B622" s="5"/>
       <c r="C622" s="5"/>
@@ -25664,27 +25668,47 @@
       <c r="O622" s="5"/>
       <c r="P622" s="5"/>
     </row>
+    <row r="623" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A623" s="5" t="s">
+        <v>833</v>
+      </c>
+      <c r="B623" s="5"/>
+      <c r="C623" s="5"/>
+      <c r="D623" s="5"/>
+      <c r="E623" s="5"/>
+      <c r="F623" s="5"/>
+      <c r="G623" s="5"/>
+      <c r="H623" s="5"/>
+      <c r="I623" s="5"/>
+      <c r="J623" s="5"/>
+      <c r="K623" s="5"/>
+      <c r="L623" s="5"/>
+      <c r="M623" s="5"/>
+      <c r="N623" s="5"/>
+      <c r="O623" s="5"/>
+      <c r="P623" s="5"/>
+    </row>
     <row r="624" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A624" s="42" t="s">
+      <c r="A624" s="5" t="s">
         <v>834</v>
       </c>
-      <c r="B624" s="42"/>
-      <c r="C624" s="42"/>
-      <c r="D624" s="42"/>
-      <c r="E624" s="42"/>
-      <c r="F624" s="42"/>
-      <c r="G624" s="42"/>
-      <c r="H624" s="42"/>
-      <c r="I624" s="42"/>
-      <c r="J624" s="42"/>
-      <c r="K624" s="42"/>
-      <c r="L624" s="42"/>
-      <c r="M624" s="42"/>
-      <c r="N624" s="42"/>
-      <c r="O624" s="42"/>
-      <c r="P624" s="42"/>
-    </row>
-    <row r="625" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B624" s="5"/>
+      <c r="C624" s="5"/>
+      <c r="D624" s="5"/>
+      <c r="E624" s="5"/>
+      <c r="F624" s="5"/>
+      <c r="G624" s="5"/>
+      <c r="H624" s="5"/>
+      <c r="I624" s="5"/>
+      <c r="J624" s="5"/>
+      <c r="K624" s="5"/>
+      <c r="L624" s="5"/>
+      <c r="M624" s="5"/>
+      <c r="N624" s="5"/>
+      <c r="O624" s="5"/>
+      <c r="P624" s="5"/>
+    </row>
+    <row r="625" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A625" s="5" t="s">
         <v>835</v>
       </c>
@@ -25704,7 +25728,7 @@
       <c r="O625" s="5"/>
       <c r="P625" s="5"/>
     </row>
-    <row r="626" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="626" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A626" s="5" t="s">
         <v>836</v>
       </c>
@@ -25724,7 +25748,7 @@
       <c r="O626" s="5"/>
       <c r="P626" s="5"/>
     </row>
-    <row r="627" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="627" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A627" s="5" t="s">
         <v>837</v>
       </c>
@@ -25784,45 +25808,45 @@
       <c r="O629" s="5"/>
       <c r="P629" s="5"/>
     </row>
-    <row r="630" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A630" s="5" t="s">
+    <row r="631" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A631" s="42" t="s">
         <v>840</v>
       </c>
-      <c r="B630" s="5"/>
-      <c r="C630" s="5"/>
-      <c r="D630" s="5"/>
-      <c r="E630" s="5"/>
-      <c r="F630" s="5"/>
-      <c r="G630" s="5"/>
-      <c r="H630" s="5"/>
-      <c r="I630" s="5"/>
-      <c r="J630" s="5"/>
-      <c r="K630" s="5"/>
-      <c r="L630" s="5"/>
-      <c r="M630" s="5"/>
-      <c r="N630" s="5"/>
-      <c r="O630" s="5"/>
-      <c r="P630" s="5"/>
-    </row>
-    <row r="632" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A632" s="42" t="s">
+      <c r="B631" s="42"/>
+      <c r="C631" s="42"/>
+      <c r="D631" s="42"/>
+      <c r="E631" s="42"/>
+      <c r="F631" s="42"/>
+      <c r="G631" s="42"/>
+      <c r="H631" s="42"/>
+      <c r="I631" s="42"/>
+      <c r="J631" s="42"/>
+      <c r="K631" s="42"/>
+      <c r="L631" s="42"/>
+      <c r="M631" s="42"/>
+      <c r="N631" s="42"/>
+      <c r="O631" s="42"/>
+      <c r="P631" s="42"/>
+    </row>
+    <row r="632" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A632" s="5" t="s">
         <v>841</v>
       </c>
-      <c r="B632" s="42"/>
-      <c r="C632" s="42"/>
-      <c r="D632" s="42"/>
-      <c r="E632" s="42"/>
-      <c r="F632" s="42"/>
-      <c r="G632" s="42"/>
-      <c r="H632" s="42"/>
-      <c r="I632" s="42"/>
-      <c r="J632" s="42"/>
-      <c r="K632" s="42"/>
-      <c r="L632" s="42"/>
-      <c r="M632" s="42"/>
-      <c r="N632" s="42"/>
-      <c r="O632" s="42"/>
-      <c r="P632" s="42"/>
+      <c r="B632" s="5"/>
+      <c r="C632" s="5"/>
+      <c r="D632" s="5"/>
+      <c r="E632" s="5"/>
+      <c r="F632" s="5"/>
+      <c r="G632" s="5"/>
+      <c r="H632" s="5"/>
+      <c r="I632" s="5"/>
+      <c r="J632" s="5"/>
+      <c r="K632" s="5"/>
+      <c r="L632" s="5"/>
+      <c r="M632" s="5"/>
+      <c r="N632" s="5"/>
+      <c r="O632" s="5"/>
+      <c r="P632" s="5"/>
     </row>
     <row r="633" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A633" s="5" t="s">
@@ -25844,7 +25868,7 @@
       <c r="O633" s="5"/>
       <c r="P633" s="5"/>
     </row>
-    <row r="634" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="634" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A634" s="5" t="s">
         <v>843</v>
       </c>
@@ -25924,49 +25948,29 @@
       <c r="O637" s="5"/>
       <c r="P637" s="5"/>
     </row>
-    <row r="638" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A638" s="5" t="s">
+    <row r="639" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A639" s="42" t="s">
         <v>847</v>
       </c>
-      <c r="B638" s="5"/>
-      <c r="C638" s="5"/>
-      <c r="D638" s="5"/>
-      <c r="E638" s="5"/>
-      <c r="F638" s="5"/>
-      <c r="G638" s="5"/>
-      <c r="H638" s="5"/>
-      <c r="I638" s="5"/>
-      <c r="J638" s="5"/>
-      <c r="K638" s="5"/>
-      <c r="L638" s="5"/>
-      <c r="M638" s="5"/>
-      <c r="N638" s="5"/>
-      <c r="O638" s="5"/>
-      <c r="P638" s="5"/>
-    </row>
-    <row r="639" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A639" s="5" t="s">
-        <v>848</v>
-      </c>
-      <c r="B639" s="5"/>
-      <c r="C639" s="5"/>
-      <c r="D639" s="5"/>
-      <c r="E639" s="5"/>
-      <c r="F639" s="5"/>
-      <c r="G639" s="5"/>
-      <c r="H639" s="5"/>
-      <c r="I639" s="5"/>
-      <c r="J639" s="5"/>
-      <c r="K639" s="5"/>
-      <c r="L639" s="5"/>
-      <c r="M639" s="5"/>
-      <c r="N639" s="5"/>
-      <c r="O639" s="5"/>
-      <c r="P639" s="5"/>
+      <c r="B639" s="42"/>
+      <c r="C639" s="42"/>
+      <c r="D639" s="42"/>
+      <c r="E639" s="42"/>
+      <c r="F639" s="42"/>
+      <c r="G639" s="42"/>
+      <c r="H639" s="42"/>
+      <c r="I639" s="42"/>
+      <c r="J639" s="42"/>
+      <c r="K639" s="42"/>
+      <c r="L639" s="42"/>
+      <c r="M639" s="42"/>
+      <c r="N639" s="42"/>
+      <c r="O639" s="42"/>
+      <c r="P639" s="42"/>
     </row>
     <row r="640" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A640" s="5" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B640" s="5"/>
       <c r="C640" s="5"/>
@@ -25986,7 +25990,7 @@
     </row>
     <row r="641" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A641" s="5" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B641" s="5"/>
       <c r="C641" s="5"/>
@@ -26006,7 +26010,7 @@
     </row>
     <row r="642" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A642" s="5" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B642" s="5"/>
       <c r="C642" s="5"/>
@@ -26026,7 +26030,7 @@
     </row>
     <row r="643" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A643" s="5" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B643" s="5"/>
       <c r="C643" s="5"/>
@@ -26046,7 +26050,7 @@
     </row>
     <row r="644" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A644" s="5" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B644" s="5"/>
       <c r="C644" s="5"/>
@@ -26064,9 +26068,9 @@
       <c r="O644" s="5"/>
       <c r="P644" s="5"/>
     </row>
-    <row r="645" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="645" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A645" s="5" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B645" s="5"/>
       <c r="C645" s="5"/>
@@ -26086,7 +26090,7 @@
     </row>
     <row r="646" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A646" s="5" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="B646" s="5"/>
       <c r="C646" s="5"/>
@@ -26106,7 +26110,7 @@
     </row>
     <row r="647" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A647" s="5" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B647" s="5"/>
       <c r="C647" s="5"/>
@@ -26126,7 +26130,7 @@
     </row>
     <row r="648" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A648" s="5" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B648" s="5"/>
       <c r="C648" s="5"/>
@@ -26144,27 +26148,47 @@
       <c r="O648" s="5"/>
       <c r="P648" s="5"/>
     </row>
-    <row r="650" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A650" s="42" t="s">
+    <row r="649" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A649" s="5" t="s">
+        <v>857</v>
+      </c>
+      <c r="B649" s="5"/>
+      <c r="C649" s="5"/>
+      <c r="D649" s="5"/>
+      <c r="E649" s="5"/>
+      <c r="F649" s="5"/>
+      <c r="G649" s="5"/>
+      <c r="H649" s="5"/>
+      <c r="I649" s="5"/>
+      <c r="J649" s="5"/>
+      <c r="K649" s="5"/>
+      <c r="L649" s="5"/>
+      <c r="M649" s="5"/>
+      <c r="N649" s="5"/>
+      <c r="O649" s="5"/>
+      <c r="P649" s="5"/>
+    </row>
+    <row r="650" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A650" s="5" t="s">
         <v>858</v>
       </c>
-      <c r="B650" s="42"/>
-      <c r="C650" s="42"/>
-      <c r="D650" s="42"/>
-      <c r="E650" s="42"/>
-      <c r="F650" s="42"/>
-      <c r="G650" s="42"/>
-      <c r="H650" s="42"/>
-      <c r="I650" s="42"/>
-      <c r="J650" s="42"/>
-      <c r="K650" s="42"/>
-      <c r="L650" s="42"/>
-      <c r="M650" s="42"/>
-      <c r="N650" s="42"/>
-      <c r="O650" s="42"/>
-      <c r="P650" s="42"/>
-    </row>
-    <row r="651" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B650" s="5"/>
+      <c r="C650" s="5"/>
+      <c r="D650" s="5"/>
+      <c r="E650" s="5"/>
+      <c r="F650" s="5"/>
+      <c r="G650" s="5"/>
+      <c r="H650" s="5"/>
+      <c r="I650" s="5"/>
+      <c r="J650" s="5"/>
+      <c r="K650" s="5"/>
+      <c r="L650" s="5"/>
+      <c r="M650" s="5"/>
+      <c r="N650" s="5"/>
+      <c r="O650" s="5"/>
+      <c r="P650" s="5"/>
+    </row>
+    <row r="651" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A651" s="5" t="s">
         <v>859</v>
       </c>
@@ -26184,7 +26208,7 @@
       <c r="O651" s="5"/>
       <c r="P651" s="5"/>
     </row>
-    <row r="652" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="652" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A652" s="5" t="s">
         <v>860</v>
       </c>
@@ -26204,7 +26228,7 @@
       <c r="O652" s="5"/>
       <c r="P652" s="5"/>
     </row>
-    <row r="653" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="653" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A653" s="5" t="s">
         <v>861</v>
       </c>
@@ -26224,7 +26248,7 @@
       <c r="O653" s="5"/>
       <c r="P653" s="5"/>
     </row>
-    <row r="654" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="654" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A654" s="5" t="s">
         <v>862</v>
       </c>
@@ -26244,7 +26268,7 @@
       <c r="O654" s="5"/>
       <c r="P654" s="5"/>
     </row>
-    <row r="655" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="655" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A655" s="5" t="s">
         <v>863</v>
       </c>
@@ -26264,7 +26288,7 @@
       <c r="O655" s="5"/>
       <c r="P655" s="5"/>
     </row>
-    <row r="656" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="656" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A656" s="5" t="s">
         <v>864</v>
       </c>
@@ -26284,7 +26308,7 @@
       <c r="O656" s="5"/>
       <c r="P656" s="5"/>
     </row>
-    <row r="657" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="657" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A657" s="5" t="s">
         <v>865</v>
       </c>
@@ -26304,49 +26328,29 @@
       <c r="O657" s="5"/>
       <c r="P657" s="5"/>
     </row>
-    <row r="658" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A658" s="5" t="s">
+    <row r="659" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A659" s="42" t="s">
         <v>866</v>
       </c>
-      <c r="B658" s="5"/>
-      <c r="C658" s="5"/>
-      <c r="D658" s="5"/>
-      <c r="E658" s="5"/>
-      <c r="F658" s="5"/>
-      <c r="G658" s="5"/>
-      <c r="H658" s="5"/>
-      <c r="I658" s="5"/>
-      <c r="J658" s="5"/>
-      <c r="K658" s="5"/>
-      <c r="L658" s="5"/>
-      <c r="M658" s="5"/>
-      <c r="N658" s="5"/>
-      <c r="O658" s="5"/>
-      <c r="P658" s="5"/>
-    </row>
-    <row r="659" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A659" s="5" t="s">
-        <v>867</v>
-      </c>
-      <c r="B659" s="5"/>
-      <c r="C659" s="5"/>
-      <c r="D659" s="5"/>
-      <c r="E659" s="5"/>
-      <c r="F659" s="5"/>
-      <c r="G659" s="5"/>
-      <c r="H659" s="5"/>
-      <c r="I659" s="5"/>
-      <c r="J659" s="5"/>
-      <c r="K659" s="5"/>
-      <c r="L659" s="5"/>
-      <c r="M659" s="5"/>
-      <c r="N659" s="5"/>
-      <c r="O659" s="5"/>
-      <c r="P659" s="5"/>
+      <c r="B659" s="42"/>
+      <c r="C659" s="42"/>
+      <c r="D659" s="42"/>
+      <c r="E659" s="42"/>
+      <c r="F659" s="42"/>
+      <c r="G659" s="42"/>
+      <c r="H659" s="42"/>
+      <c r="I659" s="42"/>
+      <c r="J659" s="42"/>
+      <c r="K659" s="42"/>
+      <c r="L659" s="42"/>
+      <c r="M659" s="42"/>
+      <c r="N659" s="42"/>
+      <c r="O659" s="42"/>
+      <c r="P659" s="42"/>
     </row>
     <row r="660" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A660" s="5" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B660" s="5"/>
       <c r="C660" s="5"/>
@@ -26364,9 +26368,9 @@
       <c r="O660" s="5"/>
       <c r="P660" s="5"/>
     </row>
-    <row r="661" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="661" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A661" s="5" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B661" s="5"/>
       <c r="C661" s="5"/>
@@ -26384,9 +26388,9 @@
       <c r="O661" s="5"/>
       <c r="P661" s="5"/>
     </row>
-    <row r="662" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="662" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A662" s="5" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B662" s="5"/>
       <c r="C662" s="5"/>
@@ -26404,9 +26408,9 @@
       <c r="O662" s="5"/>
       <c r="P662" s="5"/>
     </row>
-    <row r="663" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="663" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A663" s="5" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B663" s="5"/>
       <c r="C663" s="5"/>
@@ -26424,9 +26428,9 @@
       <c r="O663" s="5"/>
       <c r="P663" s="5"/>
     </row>
-    <row r="664" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="664" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A664" s="5" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B664" s="5"/>
       <c r="C664" s="5"/>
@@ -26446,7 +26450,7 @@
     </row>
     <row r="665" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A665" s="5" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="B665" s="5"/>
       <c r="C665" s="5"/>
@@ -26466,7 +26470,7 @@
     </row>
     <row r="666" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A666" s="5" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="B666" s="5"/>
       <c r="C666" s="5"/>
@@ -26484,9 +26488,9 @@
       <c r="O666" s="5"/>
       <c r="P666" s="5"/>
     </row>
-    <row r="667" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="667" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A667" s="5" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B667" s="5"/>
       <c r="C667" s="5"/>
@@ -26504,9 +26508,9 @@
       <c r="O667" s="5"/>
       <c r="P667" s="5"/>
     </row>
-    <row r="668" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="668" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A668" s="5" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B668" s="5"/>
       <c r="C668" s="5"/>
@@ -26524,9 +26528,9 @@
       <c r="O668" s="5"/>
       <c r="P668" s="5"/>
     </row>
-    <row r="669" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="669" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A669" s="5" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B669" s="5"/>
       <c r="C669" s="5"/>
@@ -26546,7 +26550,7 @@
     </row>
     <row r="670" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A670" s="5" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B670" s="5"/>
       <c r="C670" s="5"/>
@@ -26566,7 +26570,7 @@
     </row>
     <row r="671" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A671" s="5" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B671" s="5"/>
       <c r="C671" s="5"/>
@@ -26584,9 +26588,9 @@
       <c r="O671" s="5"/>
       <c r="P671" s="5"/>
     </row>
-    <row r="672" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="672" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A672" s="5" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B672" s="5"/>
       <c r="C672" s="5"/>
@@ -26604,27 +26608,47 @@
       <c r="O672" s="5"/>
       <c r="P672" s="5"/>
     </row>
-    <row r="674" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A674" s="42" t="s">
+    <row r="673" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A673" s="5" t="s">
+        <v>880</v>
+      </c>
+      <c r="B673" s="5"/>
+      <c r="C673" s="5"/>
+      <c r="D673" s="5"/>
+      <c r="E673" s="5"/>
+      <c r="F673" s="5"/>
+      <c r="G673" s="5"/>
+      <c r="H673" s="5"/>
+      <c r="I673" s="5"/>
+      <c r="J673" s="5"/>
+      <c r="K673" s="5"/>
+      <c r="L673" s="5"/>
+      <c r="M673" s="5"/>
+      <c r="N673" s="5"/>
+      <c r="O673" s="5"/>
+      <c r="P673" s="5"/>
+    </row>
+    <row r="674" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A674" s="5" t="s">
         <v>881</v>
       </c>
-      <c r="B674" s="42"/>
-      <c r="C674" s="42"/>
-      <c r="D674" s="42"/>
-      <c r="E674" s="42"/>
-      <c r="F674" s="42"/>
-      <c r="G674" s="42"/>
-      <c r="H674" s="42"/>
-      <c r="I674" s="42"/>
-      <c r="J674" s="42"/>
-      <c r="K674" s="42"/>
-      <c r="L674" s="42"/>
-      <c r="M674" s="42"/>
-      <c r="N674" s="42"/>
-      <c r="O674" s="42"/>
-      <c r="P674" s="42"/>
-    </row>
-    <row r="675" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B674" s="5"/>
+      <c r="C674" s="5"/>
+      <c r="D674" s="5"/>
+      <c r="E674" s="5"/>
+      <c r="F674" s="5"/>
+      <c r="G674" s="5"/>
+      <c r="H674" s="5"/>
+      <c r="I674" s="5"/>
+      <c r="J674" s="5"/>
+      <c r="K674" s="5"/>
+      <c r="L674" s="5"/>
+      <c r="M674" s="5"/>
+      <c r="N674" s="5"/>
+      <c r="O674" s="5"/>
+      <c r="P674" s="5"/>
+    </row>
+    <row r="675" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A675" s="5" t="s">
         <v>882</v>
       </c>
@@ -26644,7 +26668,7 @@
       <c r="O675" s="5"/>
       <c r="P675" s="5"/>
     </row>
-    <row r="676" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="676" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A676" s="5" t="s">
         <v>883</v>
       </c>
@@ -26664,7 +26688,7 @@
       <c r="O676" s="5"/>
       <c r="P676" s="5"/>
     </row>
-    <row r="677" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="677" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A677" s="5" t="s">
         <v>884</v>
       </c>
@@ -26684,7 +26708,7 @@
       <c r="O677" s="5"/>
       <c r="P677" s="5"/>
     </row>
-    <row r="678" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="678" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A678" s="5" t="s">
         <v>885</v>
       </c>
@@ -26704,7 +26728,7 @@
       <c r="O678" s="5"/>
       <c r="P678" s="5"/>
     </row>
-    <row r="679" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="679" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A679" s="5" t="s">
         <v>886</v>
       </c>
@@ -26724,7 +26748,7 @@
       <c r="O679" s="5"/>
       <c r="P679" s="5"/>
     </row>
-    <row r="680" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="680" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A680" s="5" t="s">
         <v>887</v>
       </c>
@@ -26744,7 +26768,7 @@
       <c r="O680" s="5"/>
       <c r="P680" s="5"/>
     </row>
-    <row r="681" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="681" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A681" s="5" t="s">
         <v>888</v>
       </c>
@@ -26764,49 +26788,29 @@
       <c r="O681" s="5"/>
       <c r="P681" s="5"/>
     </row>
-    <row r="682" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A682" s="5" t="s">
+    <row r="683" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A683" s="42" t="s">
         <v>889</v>
       </c>
-      <c r="B682" s="5"/>
-      <c r="C682" s="5"/>
-      <c r="D682" s="5"/>
-      <c r="E682" s="5"/>
-      <c r="F682" s="5"/>
-      <c r="G682" s="5"/>
-      <c r="H682" s="5"/>
-      <c r="I682" s="5"/>
-      <c r="J682" s="5"/>
-      <c r="K682" s="5"/>
-      <c r="L682" s="5"/>
-      <c r="M682" s="5"/>
-      <c r="N682" s="5"/>
-      <c r="O682" s="5"/>
-      <c r="P682" s="5"/>
-    </row>
-    <row r="683" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A683" s="5" t="s">
-        <v>890</v>
-      </c>
-      <c r="B683" s="5"/>
-      <c r="C683" s="5"/>
-      <c r="D683" s="5"/>
-      <c r="E683" s="5"/>
-      <c r="F683" s="5"/>
-      <c r="G683" s="5"/>
-      <c r="H683" s="5"/>
-      <c r="I683" s="5"/>
-      <c r="J683" s="5"/>
-      <c r="K683" s="5"/>
-      <c r="L683" s="5"/>
-      <c r="M683" s="5"/>
-      <c r="N683" s="5"/>
-      <c r="O683" s="5"/>
-      <c r="P683" s="5"/>
+      <c r="B683" s="42"/>
+      <c r="C683" s="42"/>
+      <c r="D683" s="42"/>
+      <c r="E683" s="42"/>
+      <c r="F683" s="42"/>
+      <c r="G683" s="42"/>
+      <c r="H683" s="42"/>
+      <c r="I683" s="42"/>
+      <c r="J683" s="42"/>
+      <c r="K683" s="42"/>
+      <c r="L683" s="42"/>
+      <c r="M683" s="42"/>
+      <c r="N683" s="42"/>
+      <c r="O683" s="42"/>
+      <c r="P683" s="42"/>
     </row>
     <row r="684" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A684" s="5" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="B684" s="5"/>
       <c r="C684" s="5"/>
@@ -26826,7 +26830,7 @@
     </row>
     <row r="685" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A685" s="5" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="B685" s="5"/>
       <c r="C685" s="5"/>
@@ -26846,7 +26850,7 @@
     </row>
     <row r="686" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A686" s="5" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B686" s="5"/>
       <c r="C686" s="5"/>
@@ -26864,8 +26868,188 @@
       <c r="O686" s="5"/>
       <c r="P686" s="5"/>
     </row>
+    <row r="687" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A687" s="5" t="s">
+        <v>893</v>
+      </c>
+      <c r="B687" s="5"/>
+      <c r="C687" s="5"/>
+      <c r="D687" s="5"/>
+      <c r="E687" s="5"/>
+      <c r="F687" s="5"/>
+      <c r="G687" s="5"/>
+      <c r="H687" s="5"/>
+      <c r="I687" s="5"/>
+      <c r="J687" s="5"/>
+      <c r="K687" s="5"/>
+      <c r="L687" s="5"/>
+      <c r="M687" s="5"/>
+      <c r="N687" s="5"/>
+      <c r="O687" s="5"/>
+      <c r="P687" s="5"/>
+    </row>
+    <row r="688" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A688" s="5" t="s">
+        <v>894</v>
+      </c>
+      <c r="B688" s="5"/>
+      <c r="C688" s="5"/>
+      <c r="D688" s="5"/>
+      <c r="E688" s="5"/>
+      <c r="F688" s="5"/>
+      <c r="G688" s="5"/>
+      <c r="H688" s="5"/>
+      <c r="I688" s="5"/>
+      <c r="J688" s="5"/>
+      <c r="K688" s="5"/>
+      <c r="L688" s="5"/>
+      <c r="M688" s="5"/>
+      <c r="N688" s="5"/>
+      <c r="O688" s="5"/>
+      <c r="P688" s="5"/>
+    </row>
+    <row r="689" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A689" s="5" t="s">
+        <v>895</v>
+      </c>
+      <c r="B689" s="5"/>
+      <c r="C689" s="5"/>
+      <c r="D689" s="5"/>
+      <c r="E689" s="5"/>
+      <c r="F689" s="5"/>
+      <c r="G689" s="5"/>
+      <c r="H689" s="5"/>
+      <c r="I689" s="5"/>
+      <c r="J689" s="5"/>
+      <c r="K689" s="5"/>
+      <c r="L689" s="5"/>
+      <c r="M689" s="5"/>
+      <c r="N689" s="5"/>
+      <c r="O689" s="5"/>
+      <c r="P689" s="5"/>
+    </row>
+    <row r="690" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A690" s="5" t="s">
+        <v>896</v>
+      </c>
+      <c r="B690" s="5"/>
+      <c r="C690" s="5"/>
+      <c r="D690" s="5"/>
+      <c r="E690" s="5"/>
+      <c r="F690" s="5"/>
+      <c r="G690" s="5"/>
+      <c r="H690" s="5"/>
+      <c r="I690" s="5"/>
+      <c r="J690" s="5"/>
+      <c r="K690" s="5"/>
+      <c r="L690" s="5"/>
+      <c r="M690" s="5"/>
+      <c r="N690" s="5"/>
+      <c r="O690" s="5"/>
+      <c r="P690" s="5"/>
+    </row>
+    <row r="691" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A691" s="5" t="s">
+        <v>897</v>
+      </c>
+      <c r="B691" s="5"/>
+      <c r="C691" s="5"/>
+      <c r="D691" s="5"/>
+      <c r="E691" s="5"/>
+      <c r="F691" s="5"/>
+      <c r="G691" s="5"/>
+      <c r="H691" s="5"/>
+      <c r="I691" s="5"/>
+      <c r="J691" s="5"/>
+      <c r="K691" s="5"/>
+      <c r="L691" s="5"/>
+      <c r="M691" s="5"/>
+      <c r="N691" s="5"/>
+      <c r="O691" s="5"/>
+      <c r="P691" s="5"/>
+    </row>
+    <row r="692" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A692" s="5" t="s">
+        <v>898</v>
+      </c>
+      <c r="B692" s="5"/>
+      <c r="C692" s="5"/>
+      <c r="D692" s="5"/>
+      <c r="E692" s="5"/>
+      <c r="F692" s="5"/>
+      <c r="G692" s="5"/>
+      <c r="H692" s="5"/>
+      <c r="I692" s="5"/>
+      <c r="J692" s="5"/>
+      <c r="K692" s="5"/>
+      <c r="L692" s="5"/>
+      <c r="M692" s="5"/>
+      <c r="N692" s="5"/>
+      <c r="O692" s="5"/>
+      <c r="P692" s="5"/>
+    </row>
+    <row r="693" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A693" s="5" t="s">
+        <v>899</v>
+      </c>
+      <c r="B693" s="5"/>
+      <c r="C693" s="5"/>
+      <c r="D693" s="5"/>
+      <c r="E693" s="5"/>
+      <c r="F693" s="5"/>
+      <c r="G693" s="5"/>
+      <c r="H693" s="5"/>
+      <c r="I693" s="5"/>
+      <c r="J693" s="5"/>
+      <c r="K693" s="5"/>
+      <c r="L693" s="5"/>
+      <c r="M693" s="5"/>
+      <c r="N693" s="5"/>
+      <c r="O693" s="5"/>
+      <c r="P693" s="5"/>
+    </row>
+    <row r="694" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A694" s="5" t="s">
+        <v>900</v>
+      </c>
+      <c r="B694" s="5"/>
+      <c r="C694" s="5"/>
+      <c r="D694" s="5"/>
+      <c r="E694" s="5"/>
+      <c r="F694" s="5"/>
+      <c r="G694" s="5"/>
+      <c r="H694" s="5"/>
+      <c r="I694" s="5"/>
+      <c r="J694" s="5"/>
+      <c r="K694" s="5"/>
+      <c r="L694" s="5"/>
+      <c r="M694" s="5"/>
+      <c r="N694" s="5"/>
+      <c r="O694" s="5"/>
+      <c r="P694" s="5"/>
+    </row>
+    <row r="695" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A695" s="5" t="s">
+        <v>901</v>
+      </c>
+      <c r="B695" s="5"/>
+      <c r="C695" s="5"/>
+      <c r="D695" s="5"/>
+      <c r="E695" s="5"/>
+      <c r="F695" s="5"/>
+      <c r="G695" s="5"/>
+      <c r="H695" s="5"/>
+      <c r="I695" s="5"/>
+      <c r="J695" s="5"/>
+      <c r="K695" s="5"/>
+      <c r="L695" s="5"/>
+      <c r="M695" s="5"/>
+      <c r="N695" s="5"/>
+      <c r="O695" s="5"/>
+      <c r="P695" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="164">
+  <mergeCells count="172">
     <mergeCell ref="A5:P5"/>
     <mergeCell ref="A6:P6"/>
     <mergeCell ref="A7:P7"/>
@@ -26925,7 +27109,6 @@
     <mergeCell ref="A574:P574"/>
     <mergeCell ref="A575:P575"/>
     <mergeCell ref="A576:P576"/>
-    <mergeCell ref="A577:P577"/>
     <mergeCell ref="A578:P578"/>
     <mergeCell ref="A579:P579"/>
     <mergeCell ref="A580:P580"/>
@@ -26937,13 +27120,13 @@
     <mergeCell ref="A586:P586"/>
     <mergeCell ref="A587:P587"/>
     <mergeCell ref="A588:P588"/>
+    <mergeCell ref="A589:P589"/>
     <mergeCell ref="A590:P590"/>
     <mergeCell ref="A591:P591"/>
     <mergeCell ref="A592:P592"/>
     <mergeCell ref="A593:P593"/>
     <mergeCell ref="A594:P594"/>
     <mergeCell ref="A595:P595"/>
-    <mergeCell ref="A596:P596"/>
     <mergeCell ref="A597:P597"/>
     <mergeCell ref="A598:P598"/>
     <mergeCell ref="A599:P599"/>
@@ -26970,20 +27153,20 @@
     <mergeCell ref="A620:P620"/>
     <mergeCell ref="A621:P621"/>
     <mergeCell ref="A622:P622"/>
+    <mergeCell ref="A623:P623"/>
     <mergeCell ref="A624:P624"/>
     <mergeCell ref="A625:P625"/>
     <mergeCell ref="A626:P626"/>
     <mergeCell ref="A627:P627"/>
     <mergeCell ref="A628:P628"/>
     <mergeCell ref="A629:P629"/>
-    <mergeCell ref="A630:P630"/>
+    <mergeCell ref="A631:P631"/>
     <mergeCell ref="A632:P632"/>
     <mergeCell ref="A633:P633"/>
     <mergeCell ref="A634:P634"/>
     <mergeCell ref="A635:P635"/>
     <mergeCell ref="A636:P636"/>
     <mergeCell ref="A637:P637"/>
-    <mergeCell ref="A638:P638"/>
     <mergeCell ref="A639:P639"/>
     <mergeCell ref="A640:P640"/>
     <mergeCell ref="A641:P641"/>
@@ -26994,6 +27177,7 @@
     <mergeCell ref="A646:P646"/>
     <mergeCell ref="A647:P647"/>
     <mergeCell ref="A648:P648"/>
+    <mergeCell ref="A649:P649"/>
     <mergeCell ref="A650:P650"/>
     <mergeCell ref="A651:P651"/>
     <mergeCell ref="A652:P652"/>
@@ -27002,7 +27186,6 @@
     <mergeCell ref="A655:P655"/>
     <mergeCell ref="A656:P656"/>
     <mergeCell ref="A657:P657"/>
-    <mergeCell ref="A658:P658"/>
     <mergeCell ref="A659:P659"/>
     <mergeCell ref="A660:P660"/>
     <mergeCell ref="A661:P661"/>
@@ -27017,6 +27200,7 @@
     <mergeCell ref="A670:P670"/>
     <mergeCell ref="A671:P671"/>
     <mergeCell ref="A672:P672"/>
+    <mergeCell ref="A673:P673"/>
     <mergeCell ref="A674:P674"/>
     <mergeCell ref="A675:P675"/>
     <mergeCell ref="A676:P676"/>
@@ -27025,11 +27209,19 @@
     <mergeCell ref="A679:P679"/>
     <mergeCell ref="A680:P680"/>
     <mergeCell ref="A681:P681"/>
-    <mergeCell ref="A682:P682"/>
     <mergeCell ref="A683:P683"/>
     <mergeCell ref="A684:P684"/>
     <mergeCell ref="A685:P685"/>
     <mergeCell ref="A686:P686"/>
+    <mergeCell ref="A687:P687"/>
+    <mergeCell ref="A688:P688"/>
+    <mergeCell ref="A689:P689"/>
+    <mergeCell ref="A690:P690"/>
+    <mergeCell ref="A691:P691"/>
+    <mergeCell ref="A692:P692"/>
+    <mergeCell ref="A693:P693"/>
+    <mergeCell ref="A694:P694"/>
+    <mergeCell ref="A695:P695"/>
   </mergeCells>
   <conditionalFormatting sqref="B155:F159">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">

</xml_diff>